<commit_message>
WIP: stage current main changes before merging branches
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/quotes.xlsx
+++ b/quotes.xlsx
@@ -4208,8 +4208,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H92" s="2" t="inlineStr"/>
-      <c r="I92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>18462591727105710</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="100" customHeight="1">
       <c r="A93" s="2" t="n">

</xml_diff>

<commit_message>
Spec: Jamendo music-source swap (replace dead Pixabay music API)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/quotes.xlsx
+++ b/quotes.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audience Guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Quotes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Audience Guide" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9208,8 +9208,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H220" s="2" t="inlineStr"/>
-      <c r="I220" s="2" t="inlineStr"/>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t>18142151905548599</t>
+        </is>
+      </c>
     </row>
     <row r="221" ht="100" customHeight="1">
       <c r="A221" s="2" t="n">

</xml_diff>

<commit_message>
Spec: viral-formula generators (B) + Trend Scout (NEW)
Two coupled sub-projects: B adds formula-compliant hook/CTA/caption/hashtag
generators, a --content injection path, and an optional Remotion BridgeScene;
NEW adds a Trend Scout agent that sources live trends (Google Trends + GNews),
picks the safest-bridging one, and injects a trending hook + bridge.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/quotes.xlsx
+++ b/quotes.xlsx
@@ -9333,8 +9333,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H223" s="2" t="inlineStr"/>
-      <c r="I223" s="2" t="inlineStr"/>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>18096924953153801</t>
+        </is>
+      </c>
     </row>
     <row r="224" ht="100" customHeight="1">
       <c r="A224" s="2" t="n">

</xml_diff>

<commit_message>
Plan: Trend Scout (4 tasks, TDD)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/quotes.xlsx
+++ b/quotes.xlsx
@@ -9497,8 +9497,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H227" s="2" t="inlineStr"/>
-      <c r="I227" s="2" t="inlineStr"/>
+      <c r="H227" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>18022119059683452</t>
+        </is>
+      </c>
     </row>
     <row r="228" ht="100" customHeight="1">
       <c r="A228" s="2" t="n">

</xml_diff>

<commit_message>
sync tracked working changes: sdd reports, reel-data, landing, notifications, quotes
- update task-1..9 sdd reports/briefs
- reel-data.json content additions
- landing.html tweaks
- notifications log append
- quotes.xlsx refresh

untracked bg*.mp4 + .hermes/ skipped per request
</commit_message>
<xml_diff>
--- a/quotes.xlsx
+++ b/quotes.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Quotes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Audience Guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audience Guide" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2297,8 +2297,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr"/>
-      <c r="I43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>17960555829149408</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="100" customHeight="1">
       <c r="A44" s="2" t="n">
@@ -10285,8 +10293,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H247" s="2" t="inlineStr"/>
-      <c r="I247" s="2" t="inlineStr"/>
+      <c r="H247" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>18030818942826689</t>
+        </is>
+      </c>
     </row>
     <row r="248" ht="100" customHeight="1">
       <c r="A248" s="2" t="n">
@@ -10363,8 +10379,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H249" s="2" t="inlineStr"/>
-      <c r="I249" s="2" t="inlineStr"/>
+      <c r="H249" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I249" s="2" t="inlineStr">
+        <is>
+          <t>18107147885100723</t>
+        </is>
+      </c>
     </row>
     <row r="250" ht="100" customHeight="1">
       <c r="A250" s="2" t="n">
@@ -10558,8 +10582,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H254" s="2" t="inlineStr"/>
-      <c r="I254" s="2" t="inlineStr"/>
+      <c r="H254" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I254" s="2" t="inlineStr">
+        <is>
+          <t>18181068541406262</t>
+        </is>
+      </c>
     </row>
     <row r="255" ht="100" customHeight="1">
       <c r="A255" s="2" t="n">
@@ -10714,8 +10746,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H258" s="2" t="inlineStr"/>
-      <c r="I258" s="2" t="inlineStr"/>
+      <c r="H258" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="I258" s="2" t="inlineStr">
+        <is>
+          <t>18452110864141345</t>
+        </is>
+      </c>
     </row>
     <row r="259" ht="100" customHeight="1">
       <c r="A259" s="2" t="n">
@@ -10831,8 +10871,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H261" s="2" t="inlineStr"/>
-      <c r="I261" s="2" t="inlineStr"/>
+      <c r="H261" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="I261" s="2" t="inlineStr">
+        <is>
+          <t>18060180893767472</t>
+        </is>
+      </c>
     </row>
     <row r="262" ht="100" customHeight="1">
       <c r="A262" s="2" t="n">

</xml_diff>

<commit_message>
feat(hyperframes): Python bridge tests + shared sceneFrames + pipeline renderer dispatch fixes
</commit_message>
<xml_diff>
--- a/quotes.xlsx
+++ b/quotes.xlsx
@@ -11776,8 +11776,16 @@
           <t>ready</t>
         </is>
       </c>
-      <c r="H284" s="2" t="inlineStr"/>
-      <c r="I284" s="2" t="inlineStr"/>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="I284" s="2" t="inlineStr">
+        <is>
+          <t>18088048217359747</t>
+        </is>
+      </c>
     </row>
     <row r="285" ht="100" customHeight="1">
       <c r="A285" s="2" t="n">

</xml_diff>